<commit_message>
📊 Horarios actualizados Línea 141 - 4082
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:08:16</t>
+          <t>Última actualización: 02:15:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01:08:16</t>
+          <t>02:15:14</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01:25</t>
+          <t>03:02</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,23 +498,48 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>01:08:16</t>
+          <t>02:15:14</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:02</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>114</v>
+        <v>93</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>02:15:14</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>04:02</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>107</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -544,7 +569,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:08:16</t>
+          <t>Última actualización: 02:15:14</t>
         </is>
       </c>
     </row>
@@ -579,7 +604,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:08:16</t>
+          <t>Última actualización: 02:15:14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4083
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:15:14</t>
+          <t>Última actualización: 02:57:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -473,12 +473,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:15:14</t>
+          <t>02:57:51</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:02</t>
+          <t>03:01</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>47</v>
+        <v>4</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,7 +498,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:15:14</t>
+          <t>02:57:51</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>93</v>
+        <v>51</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,12 +523,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:15:14</t>
+          <t>02:57:51</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:02</t>
+          <t>04:01</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -537,9 +537,59 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>107</v>
+        <v>64</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>02:57:51</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>04:47</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>110</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>02:57:51</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>04:53</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>116</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -569,7 +619,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:15:14</t>
+          <t>Última actualización: 02:57:51</t>
         </is>
       </c>
     </row>
@@ -604,7 +654,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:15:14</t>
+          <t>Última actualización: 02:57:51</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4084
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:57:51</t>
+          <t>Última actualización: 03:46:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:57:51</t>
+          <t>03:46:44</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:01</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:57:51</t>
+          <t>03:46:44</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>04:01</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,12 +523,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:57:51</t>
+          <t>03:46:44</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:01</t>
+          <t>04:47</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>02:57:51</t>
+          <t>03:46:44</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04:47</t>
+          <t>04:53</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>110</v>
+        <v>67</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,23 +573,73 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>02:57:51</t>
+          <t>03:46:44</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:16</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>116</v>
+        <v>90</v>
       </c>
       <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>03:46:44</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>05:22</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>96</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>03:46:44</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>05:44</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>118</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -619,7 +669,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:57:51</t>
+          <t>Última actualización: 03:46:44</t>
         </is>
       </c>
     </row>
@@ -654,7 +704,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:57:51</t>
+          <t>Última actualización: 03:46:44</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4085
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:46:44</t>
+          <t>Última actualización: 04:40:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03:46:44</t>
+          <t>04:40:34</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>04:47</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>03:46:44</t>
+          <t>04:40:34</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:01</t>
+          <t>04:53</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>03:46:44</t>
+          <t>04:40:34</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:47</t>
+          <t>05:17</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>61</v>
+        <v>37</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>03:46:44</t>
+          <t>04:40:34</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>67</v>
+        <v>42</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>03:46:44</t>
+          <t>04:40:34</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:16</t>
+          <t>05:44</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>90</v>
+        <v>64</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>03:46:44</t>
+          <t>04:40:34</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>05:47</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>96</v>
+        <v>67</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,23 +623,173 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>03:46:44</t>
+          <t>04:40:34</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>06:01</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>118</v>
+        <v>81</v>
       </c>
       <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>04:40:34</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06:09</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>89</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>04:40:34</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>92</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>04:40:34</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>110</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>04:40:34</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>06:34</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>114</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>04:40:34</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>119</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>04:40:34</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>119</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -656,7 +806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -669,14 +819,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:46:44</t>
+          <t>Última actualización: 04:40:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>04:40:34</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>92</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -704,7 +906,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:46:44</t>
+          <t>Última actualización: 04:40:34</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4086
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:40:34</t>
+          <t>Última actualización: 05:23:42</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:40:34</t>
+          <t>05:23:42</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:47</t>
+          <t>05:23</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:40:34</t>
+          <t>05:23:42</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:44</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:40:34</t>
+          <t>05:23:42</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:17</t>
+          <t>05:47</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:40:34</t>
+          <t>05:23:42</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>06:09</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:40:34</t>
+          <t>05:23:42</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,17 +598,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:40:34</t>
+          <t>05:23:42</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:40:34</t>
+          <t>05:23:42</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>06:36</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:40:34</t>
+          <t>05:23:42</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:40:34</t>
+          <t>05:23:42</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>04:40:34</t>
+          <t>05:23:42</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>110</v>
+        <v>78</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04:40:34</t>
+          <t>05:23:42</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06:34</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>114</v>
+        <v>96</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04:40:34</t>
+          <t>05:23:42</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>07:02</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>119</v>
+        <v>99</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>04:40:34</t>
+          <t>05:23:42</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -819,14 +819,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:40:34</t>
+          <t>Última actualización: 05:23:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 2</t>
         </is>
       </c>
     </row>
@@ -860,7 +860,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:40:34</t>
+          <t>05:23:42</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -874,9 +874,34 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>92</v>
+        <v>49</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>05:23:42</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>99</v>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -906,7 +931,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:40:34</t>
+          <t>Última actualización: 05:23:42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4087
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:23:42</t>
+          <t>Última actualización: 06:07:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:23:42</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05:23</t>
+          <t>06:09</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:23:42</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:23:42</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05:23:42</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>06:36</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:23:42</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05:23:42</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>67</v>
+        <v>33</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:23:42</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:36</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>73</v>
+        <v>33</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:23:42</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>76</v>
+        <v>52</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:23:42</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:40</t>
+          <t>07:02</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>77</v>
+        <v>55</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>05:23:42</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:23:42</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>96</v>
+        <v>79</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:23:42</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:02</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>99</v>
+        <v>79</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,23 +773,98 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>05:23:42</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>117</v>
+        <v>84</v>
       </c>
       <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>06:07:50</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>89</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>06:07:50</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>07:44</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>97</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>06:07:50</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>08:06</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>119</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -806,7 +881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -819,14 +894,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:23:42</t>
+          <t>Última actualización: 06:07:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -860,7 +935,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:23:42</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -874,7 +949,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>49</v>
+        <v>5</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -885,7 +960,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:23:42</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -899,9 +974,34 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>99</v>
+        <v>55</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>06:07:50</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>84</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -918,7 +1018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -931,14 +1031,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:23:42</t>
+          <t>Última actualización: 06:07:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>06:07:50</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>101</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4088
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:07:50</t>
+          <t>Última actualización: 06:52:02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>06:52:02</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>52</v>
+        <v>7</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>06:52:02</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>07:03</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>73</v>
+        <v>11</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -728,16 +728,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>06:52:02</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>79</v>
+        <v>29</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -778,16 +778,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -803,16 +803,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>06:52:02</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07:44</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>97</v>
+        <v>35</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,23 +848,323 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>06:52:02</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>07:27</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>35</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>06:07:50</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>84</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>06:52:02</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>07:32</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>40</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>06:07:50</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>89</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>06:52:02</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>07:37</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>45</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>06:52:02</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>07:44</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>52</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>06:52:02</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>07:52</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>60</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>06:52:02</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>08:01</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>69</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>06:52:02</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
           <t>08:06</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D21" t="n">
-        <v>119</v>
-      </c>
-      <c r="E21" t="inlineStr">
+      <c r="D29" t="n">
+        <v>74</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>06:52:02</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>08:22</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>90</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>06:52:02</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>08:26</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>94</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>06:52:02</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>113</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>06:52:02</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>113</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -881,7 +1181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -894,14 +1194,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:07:50</t>
+          <t>Última actualización: 06:52:02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -985,23 +1285,148 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>06:52:02</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>07:03</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>11</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>06:07:50</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>07:31</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D9" t="n">
         <v>84</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>06:52:02</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>07:32</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>40</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>06:52:02</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>07:52</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>60</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>06:52:02</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>113</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>06:52:02</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>113</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1018,7 +1443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1031,14 +1456,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:07:50</t>
+          <t>Última actualización: 06:52:02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -1089,6 +1514,56 @@
         <v>101</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>06:52:02</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>57</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>06:52:02</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>106</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4089
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:52:02</t>
+          <t>Última actualización: 07:20:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -773,7 +773,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>79</v>
+        <v>6</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>84</v>
+        <v>11</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>89</v>
+        <v>16</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>06:52:02</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,12 +998,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:52:02</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>07:52</t>
+          <t>07:51</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>60</v>
+        <v>31</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1028,16 +1028,16 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>08:01</t>
+          <t>07:52</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,21 +1048,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>06:52:02</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>08:06</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>74</v>
+        <v>41</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,21 +1073,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>06:52:02</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:06</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>90</v>
+        <v>46</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,21 +1098,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>06:52:02</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>08:26</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>94</v>
+        <v>59</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1128,16 +1128,16 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>08:22</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,23 +1148,248 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>07:20:43</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>08:25</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>65</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>06:52:02</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>08:26</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>94</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>07:20:43</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>84</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>07:20:43</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>84</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>06:52:02</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
         <is>
           <t>08:45</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D33" t="n">
+      <c r="D37" t="n">
         <v>113</v>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>06:52:02</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>113</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>07:20:43</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>09:04</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>104</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>07:20:43</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>106</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>07:20:43</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>09:11</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>111</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>07:20:43</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>116</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1181,7 +1406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1194,14 +1419,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:52:02</t>
+          <t>Última actualización: 07:20:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1535,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1324,7 +1549,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>84</v>
+        <v>11</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1360,12 +1585,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>06:52:02</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>07:52</t>
+          <t>07:51</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1374,7 +1599,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>60</v>
+        <v>31</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1390,16 +1615,16 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>07:52</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>113</v>
+        <v>60</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1410,23 +1635,123 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>07:20:43</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>84</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>07:20:43</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>84</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>06:52:02</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>08:45</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>113</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>06:52:02</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D16" t="n">
         <v>113</v>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>07:20:43</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>106</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1443,7 +1768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1456,14 +1781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:52:02</t>
+          <t>Última actualización: 07:20:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -1497,7 +1822,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1511,7 +1836,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>101</v>
+        <v>28</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1547,25 +1872,75 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>07:20:43</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>08:37</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>77</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>06:52:02</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>08:38</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D9" t="n">
         <v>106</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>07:20:43</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>09:02</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>102</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4090
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:20:43</t>
+          <t>Última actualización: 07:58:23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 45</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -783,11 +783,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>6</v>
+        <v>79</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>79</v>
+        <v>6</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1048,7 +1048,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>07:58:23</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,7 +1073,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>07:58:23</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>07:58:23</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1112,7 +1112,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>59</v>
+        <v>21</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1148,21 +1148,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>07:58:23</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>08:25</t>
+          <t>08:23</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>65</v>
+        <v>25</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,12 +1173,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:52:02</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>08:26</t>
+          <t>08:25</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1187,7 +1187,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>94</v>
+        <v>65</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,21 +1198,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>07:58:23</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>08:44</t>
+          <t>08:26</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>84</v>
+        <v>28</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1248,21 +1248,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>06:52:02</t>
+          <t>07:58:23</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>113</v>
+        <v>46</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>07:58:23</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>09:04</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>104</v>
+        <v>47</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,21 +1323,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>07:58:23</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>08:46</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>106</v>
+        <v>48</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>07:58:23</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>09:11</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>111</v>
+        <v>66</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,23 +1373,223 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>07:58:23</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>68</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>07:58:23</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>09:11</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>73</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>07:20:43</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>09:16</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D42" t="n">
+      <c r="D44" t="n">
         <v>116</v>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>07:58:23</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>79</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>07:58:23</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>86</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>07:58:23</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>96</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>07:58:23</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>97</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>07:58:23</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>106</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>07:58:23</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>117</v>
+      </c>
+      <c r="E50" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1406,7 +1606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1419,14 +1619,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:20:43</t>
+          <t>Última actualización: 07:58:23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -1635,7 +1835,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>07:58:23</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1649,7 +1849,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>84</v>
+        <v>46</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1685,7 +1885,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>06:52:02</t>
+          <t>07:58:23</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1695,11 +1895,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>113</v>
+        <v>47</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1720,7 +1920,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1735,7 +1935,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>07:58:23</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1749,9 +1949,34 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>106</v>
+        <v>68</v>
       </c>
       <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>07:58:23</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>117</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1768,7 +1993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1781,14 +2006,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:20:43</t>
+          <t>Última actualización: 07:58:23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -1897,7 +2122,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>06:52:02</t>
+          <t>07:58:23</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1911,7 +2136,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>106</v>
+        <v>40</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1941,6 +2166,56 @@
       <c r="E10" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>07:58:23</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>09:03</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>65</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>07:58:23</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>90</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4091
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:58:23</t>
+          <t>Última actualización: 08:24:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 45</t>
+          <t>Total filas: 53</t>
         </is>
       </c>
     </row>
@@ -1173,12 +1173,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>08:25</t>
+          <t>08:24</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1187,7 +1187,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,21 +1198,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>07:58:23</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>08:26</t>
+          <t>08:24</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1228,16 +1228,16 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>08:44</t>
+          <t>08:25</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>84</v>
+        <v>65</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1253,16 +1253,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>08:44</t>
+          <t>08:26</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,21 +1273,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>06:52:02</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>08:42</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>113</v>
+        <v>18</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,12 +1298,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:58:23</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1312,7 +1312,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>47</v>
+        <v>84</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,21 +1323,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>07:58:23</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>08:46</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>07:58:23</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>09:04</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>66</v>
+        <v>21</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:58:23</t>
+          <t>06:52:02</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>68</v>
+        <v>113</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1403,16 +1403,16 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>09:11</t>
+          <t>08:46</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>73</v>
+        <v>48</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>116</v>
+        <v>40</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,21 +1448,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07:58:23</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>79</v>
+        <v>42</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,21 +1473,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>07:58:23</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>86</v>
+        <v>47</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,21 +1498,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>07:58:23</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>96</v>
+        <v>116</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,21 +1523,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>07:58:23</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>97</v>
+        <v>52</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1553,16 +1553,16 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,23 +1573,223 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>08:24:30</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>60</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>07:58:23</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>96</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>08:24:30</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>71</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>08:24:30</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>80</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>08:24:30</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>09:54</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>90</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>08:24:30</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
         <is>
           <t>09:55</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D50" t="n">
-        <v>117</v>
-      </c>
-      <c r="E50" t="inlineStr">
+      <c r="D55" t="n">
+        <v>91</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>08:24:30</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>09:59</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>95</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>08:24:30</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>106</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>08:24:30</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>111</v>
+      </c>
+      <c r="E58" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1619,7 +1819,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:58:23</t>
+          <t>Última actualización: 08:24:30</t>
         </is>
       </c>
     </row>
@@ -1835,7 +2035,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07:58:23</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1849,7 +2049,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1885,7 +2085,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>07:58:23</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1899,7 +2099,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>47</v>
+        <v>21</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1935,7 +2135,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>07:58:23</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1949,7 +2149,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>68</v>
+        <v>42</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1960,7 +2160,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>07:58:23</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1974,7 +2174,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>117</v>
+        <v>91</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1993,7 +2193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2006,14 +2206,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:58:23</t>
+          <t>Última actualización: 08:24:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2322,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07:58:23</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2136,7 +2336,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -2172,7 +2372,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07:58:23</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2186,7 +2386,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>65</v>
+        <v>39</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2197,7 +2397,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07:58:23</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2211,11 +2411,36 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>90</v>
+        <v>64</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>08:24:30</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>114</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4092
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:24:30</t>
+          <t>Última actualización: 08:52:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 53</t>
+          <t>Total filas: 63</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1462,7 +1462,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,7 +1473,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1587,7 +1587,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1623,7 +1623,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1637,7 +1637,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>71</v>
+        <v>43</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1673,21 +1673,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>09:54</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>90</v>
+        <v>53</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,21 +1698,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>09:55</t>
+          <t>09:51</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>91</v>
+        <v>59</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>09:59</t>
+          <t>09:52</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>95</v>
+        <v>60</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1753,16 +1753,16 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>10:10</t>
+          <t>09:54</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,23 +1773,273 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>08:52:08</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>63</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>08:24:30</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>09:59</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>95</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>08:52:08</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>10:01</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>69</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>08:52:08</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>72</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>08:24:30</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>106</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>08:52:08</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
         <is>
           <t>10:15</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D58" t="n">
-        <v>111</v>
-      </c>
-      <c r="E58" t="inlineStr">
+      <c r="D63" t="n">
+        <v>83</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>08:52:08</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>86</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>08:52:08</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>10:25</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>93</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>08:52:08</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>100</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>08:52:08</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>102</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>08:52:08</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>112</v>
+      </c>
+      <c r="E68" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1819,7 +2069,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:24:30</t>
+          <t>Última actualización: 08:52:08</t>
         </is>
       </c>
     </row>
@@ -2135,7 +2385,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2149,7 +2399,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2160,7 +2410,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2174,7 +2424,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>91</v>
+        <v>63</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -2193,7 +2443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2206,14 +2456,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:24:30</t>
+          <t>Última actualización: 08:52:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -2372,7 +2622,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2386,7 +2636,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2397,7 +2647,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2411,7 +2661,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>64</v>
+        <v>36</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2422,7 +2672,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2436,11 +2686,61 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>114</v>
+        <v>86</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>08:52:08</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>98</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>08:52:08</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>111</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4093
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:52:08</t>
+          <t>Última actualización: 09:23:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 63</t>
+          <t>Total filas: 71</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -833,7 +833,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1573,21 +1573,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>09:23</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,21 +1598,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>07:58:23</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:24</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>96</v>
+        <v>1</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,21 +1623,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,21 +1648,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:35</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>80</v>
+        <v>12</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,12 +1673,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>09:44</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>53</v>
+        <v>80</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1703,16 +1703,16 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>09:51</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>09:52</t>
+          <t>09:51</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,12 +1748,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>09:54</t>
+          <t>09:52</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,21 +1773,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>09:55</t>
+          <t>09:54</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>63</v>
+        <v>90</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,21 +1798,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>09:59</t>
+          <t>09:55</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>95</v>
+        <v>32</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,21 +1823,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>10:01</t>
+          <t>09:59</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>69</v>
+        <v>95</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,21 +1848,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>72</v>
+        <v>38</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,21 +1873,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>10:10</t>
+          <t>10:04</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>106</v>
+        <v>41</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,21 +1898,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>10:10</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>83</v>
+        <v>106</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,21 +1923,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>10:18</t>
+          <t>10:15</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>86</v>
+        <v>52</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1953,16 +1953,16 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>10:25</t>
+          <t>10:18</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,21 +1973,21 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>10:32</t>
+          <t>10:25</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>100</v>
+        <v>62</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,21 +1998,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>10:34</t>
+          <t>10:26</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>102</v>
+        <v>63</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2028,18 +2028,218 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>100</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>09:23:09</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>71</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>09:23:09</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
           <t>10:44</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C70" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D68" t="n">
+      <c r="D70" t="n">
+        <v>81</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>09:23:09</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>10:54</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>91</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>09:23:09</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>92</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>09:23:09</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>10:57</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>94</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>09:23:09</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>102</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>09:23:09</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>105</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>09:23:09</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
         <v>112</v>
       </c>
-      <c r="E68" t="inlineStr">
+      <c r="E76" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2069,7 +2269,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:52:08</t>
+          <t>Última actualización: 09:23:09</t>
         </is>
       </c>
     </row>
@@ -2410,7 +2610,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2424,7 +2624,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -2456,7 +2656,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:52:08</t>
+          <t>Última actualización: 09:23:09</t>
         </is>
       </c>
     </row>
@@ -2647,7 +2847,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2661,7 +2861,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>36</v>
+        <v>5</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2672,7 +2872,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2686,7 +2886,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2697,7 +2897,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2711,7 +2911,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>98</v>
+        <v>67</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2722,7 +2922,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2736,7 +2936,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>111</v>
+        <v>80</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4094
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:23:09</t>
+          <t>Última actualización: 10:27:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 71</t>
+          <t>Total filas: 90</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -783,11 +783,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>79</v>
+        <v>6</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>6</v>
+        <v>79</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -833,7 +833,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>10:27:56</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>10:32</t>
+          <t>10:28</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,21 +2048,21 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>09:23:09</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>10:34</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>71</v>
+        <v>100</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>09:23:09</t>
+          <t>10:27:56</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>10:44</t>
+          <t>10:34</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>81</v>
+        <v>7</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>09:23:09</t>
+          <t>10:27:56</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>10:54</t>
+          <t>10:43</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>91</v>
+        <v>16</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2128,16 +2128,16 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>10:55</t>
+          <t>10:44</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,21 +2148,21 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>09:23:09</t>
+          <t>10:27:56</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>10:57</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>94</v>
+        <v>24</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,21 +2173,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>09:23:09</t>
+          <t>10:27:56</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>11:05</t>
+          <t>10:54</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>102</v>
+        <v>27</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2203,16 +2203,16 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>10:54</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>105</v>
+        <v>91</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2228,18 +2228,493 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>92</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>10:27:56</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>29</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>09:23:09</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>10:57</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>94</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>10:27:56</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>11:01</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>34</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>10:27:56</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>37</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>09:23:09</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>102</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>10:27:56</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>11:07</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>40</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>09:23:09</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>105</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>10:27:56</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>11:14</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>47</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>09:23:09</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C85" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D76" t="n">
+      <c r="D85" t="n">
         <v>112</v>
       </c>
-      <c r="E76" t="inlineStr">
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>10:27:56</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>11:23</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>56</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>10:27:56</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>67</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>10:27:56</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>11:36</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>69</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>10:27:56</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>11:39</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>72</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>10:27:56</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>77</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>10:27:56</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>87</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>10:27:56</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>87</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>10:27:56</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>12:03</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>96</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>10:27:56</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>107</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>10:27:56</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>12:24</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>117</v>
+      </c>
+      <c r="E95" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2256,7 +2731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2269,14 +2744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:23:09</t>
+          <t>Última actualización: 10:27:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -2627,6 +3102,56 @@
         <v>32</v>
       </c>
       <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>10:27:56</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>67</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>10:27:56</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>77</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2643,7 +3168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2656,14 +3181,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:23:09</t>
+          <t>Última actualización: 10:27:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -2897,12 +3422,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>09:23:09</t>
+          <t>10:27:56</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>10:29</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2911,7 +3436,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>67</v>
+        <v>2</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2927,20 +3452,95 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>67</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>10:27:56</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>10:42</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>15</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>09:23:09</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>10:43</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D17" t="n">
         <v>80</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>10:27:56</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>11:22</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>55</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4095
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E95"/>
+  <dimension ref="A1:E104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:27:56</t>
+          <t>Última actualización: 11:04:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 90</t>
+          <t>Total filas: 99</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>06:52:02</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>21</v>
+        <v>113</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:52:02</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>113</v>
+        <v>21</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -2323,7 +2323,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>11:04:59</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2337,7 +2337,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>11:04:59</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>11:04:59</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2437,7 +2437,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>11:04:59</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2487,7 +2487,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>56</v>
+        <v>19</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>11:04:59</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2512,7 +2512,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>67</v>
+        <v>30</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,12 +2523,12 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>11:04:59</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>11:36</t>
+          <t>11:35</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2537,7 +2537,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>69</v>
+        <v>31</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2553,16 +2553,16 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>11:39</t>
+          <t>11:36</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2578,16 +2578,16 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>11:44</t>
+          <t>11:39</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,21 +2598,21 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>11:04:59</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>11:54</t>
+          <t>11:41</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>87</v>
+        <v>37</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,21 +2623,21 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>11:04:59</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>11:54</t>
+          <t>11:44</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>87</v>
+        <v>40</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2648,21 +2648,21 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>11:04:59</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>12:03</t>
+          <t>11:53</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>96</v>
+        <v>49</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2678,16 +2678,16 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>12:14</t>
+          <t>11:54</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>107</v>
+        <v>87</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,23 +2698,248 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>11:04:59</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>50</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>11:04:59</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>12:03</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>59</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>11:04:59</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>70</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>11:04:59</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
           <t>12:24</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
+      <c r="C98" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D95" t="n">
-        <v>117</v>
-      </c>
-      <c r="E95" t="inlineStr">
+      <c r="D98" t="n">
+        <v>80</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>11:04:59</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>12:31</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>87</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>11:04:59</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>89</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>11:04:59</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>92</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>11:04:59</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>12:43</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>99</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>11:04:59</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>101</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>11:04:59</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>110</v>
+      </c>
+      <c r="E104" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2731,7 +2956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2744,14 +2969,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:27:56</t>
+          <t>Última actualización: 11:04:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -3110,7 +3335,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>11:04:59</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3124,7 +3349,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>67</v>
+        <v>30</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -3135,7 +3360,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>11:04:59</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3149,9 +3374,34 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>77</v>
+        <v>40</v>
       </c>
       <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>11:04:59</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>110</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3181,7 +3431,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:27:56</t>
+          <t>Última actualización: 11:04:59</t>
         </is>
       </c>
     </row>
@@ -3522,7 +3772,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>11:04:59</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3536,7 +3786,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>55</v>
+        <v>18</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4096
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E104"/>
+  <dimension ref="A1:E117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:04:59</t>
+          <t>Última actualización: 11:44:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 99</t>
+          <t>Total filas: 112</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -783,11 +783,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>6</v>
+        <v>79</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>79</v>
+        <v>6</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>27</v>
+        <v>91</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>09:23:09</t>
+          <t>10:27:56</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>11:04:59</t>
+          <t>11:44:42</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2637,7 +2637,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>11:04:59</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>87</v>
+        <v>50</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>11:04:59</t>
+          <t>11:44:42</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,21 +2723,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>11:04:59</t>
+          <t>11:44:42</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>12:03</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>59</v>
+        <v>11</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2753,16 +2753,16 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>12:14</t>
+          <t>12:03</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,21 +2773,21 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>11:04:59</t>
+          <t>11:44:42</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,21 +2798,21 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>11:04:59</t>
+          <t>11:44:42</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>12:11</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>87</v>
+        <v>27</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2828,16 +2828,16 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>12:33</t>
+          <t>12:14</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,21 +2848,21 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>11:04:59</t>
+          <t>11:44:42</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>92</v>
+        <v>31</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,21 +2873,21 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>11:04:59</t>
+          <t>11:44:42</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>12:43</t>
+          <t>12:23</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>99</v>
+        <v>39</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,21 +2898,21 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>11:04:59</t>
+          <t>11:44:42</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>12:45</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>101</v>
+        <v>40</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,23 +2923,348 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
+          <t>11:44:42</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>12:31</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>47</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
           <t>11:04:59</t>
         </is>
       </c>
-      <c r="B104" t="inlineStr">
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>89</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>11:44:42</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>50</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>11:04:59</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>92</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>11:04:59</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>12:43</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>99</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>11:44:42</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>60</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>11:04:59</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>101</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>11:44:42</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>62</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>11:44:42</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
         <is>
           <t>12:54</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr">
+      <c r="C112" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D104" t="n">
-        <v>110</v>
-      </c>
-      <c r="E104" t="inlineStr">
+      <c r="D112" t="n">
+        <v>70</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>11:44:42</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>80</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>11:44:42</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>91</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>11:44:42</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>97</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>11:44:42</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>100</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>11:44:42</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>107</v>
+      </c>
+      <c r="E117" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2956,7 +3281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2969,14 +3294,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:04:59</t>
+          <t>Última actualización: 11:44:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -3185,7 +3510,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3195,11 +3520,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -3210,7 +3535,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3220,11 +3545,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -3360,7 +3685,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>11:04:59</t>
+          <t>11:44:42</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3374,7 +3699,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -3385,7 +3710,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>11:04:59</t>
+          <t>11:44:42</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3399,9 +3724,34 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>110</v>
+        <v>70</v>
       </c>
       <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>11:44:42</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>107</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3418,7 +3768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3431,14 +3781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:04:59</t>
+          <t>Última actualización: 11:44:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -3789,6 +4139,31 @@
         <v>18</v>
       </c>
       <c r="E18" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>11:44:42</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>13:22</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>98</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4097
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E117"/>
+  <dimension ref="A1:E126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:44:42</t>
+          <t>Última actualización: 12:12:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 112</t>
+          <t>Total filas: 121</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -783,11 +783,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>79</v>
+        <v>6</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>6</v>
+        <v>79</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -833,7 +833,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>11:04:59</t>
+          <t>11:44:42</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>11:44:42</t>
+          <t>11:04:59</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>11:44:42</t>
+          <t>12:12:27</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2862,7 +2862,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>31</v>
+        <v>3</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,12 +2873,12 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>11:44:42</t>
+          <t>12:12:27</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>12:23</t>
+          <t>12:19</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -2887,7 +2887,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2903,16 +2903,16 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:23</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,21 +2923,21 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>11:44:42</t>
+          <t>12:12:27</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,21 +2948,21 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>11:04:59</t>
+          <t>11:44:42</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>12:33</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>89</v>
+        <v>47</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,12 +2973,12 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>11:44:42</t>
+          <t>11:04:59</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:33</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -2987,7 +2987,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>50</v>
+        <v>89</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,21 +2998,21 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>11:04:59</t>
+          <t>12:12:27</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>92</v>
+        <v>22</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3028,16 +3028,16 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>12:43</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,21 +3048,21 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>11:44:42</t>
+          <t>12:12:27</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>12:44</t>
+          <t>12:37</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3078,16 +3078,16 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>12:45</t>
+          <t>12:43</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,21 +3098,21 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>11:44:42</t>
+          <t>12:12:27</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>12:46</t>
+          <t>12:44</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>62</v>
+        <v>32</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,21 +3123,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>11:44:42</t>
+          <t>11:04:59</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>12:54</t>
+          <t>12:45</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>70</v>
+        <v>101</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,21 +3148,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>11:44:42</t>
+          <t>12:12:27</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>12:46</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>80</v>
+        <v>34</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3178,16 +3178,16 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>91</v>
+        <v>70</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,21 +3198,21 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>11:44:42</t>
+          <t>12:12:27</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,21 +3223,21 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>11:44:42</t>
+          <t>12:12:27</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>100</v>
+        <v>52</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,23 +3248,248 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
+          <t>12:12:27</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>63</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
           <t>11:44:42</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr">
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>97</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>12:12:27</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>72</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>12:12:27</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>73</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>12:12:27</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
         <is>
           <t>13:31</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr">
+      <c r="C121" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D117" t="n">
+      <c r="D121" t="n">
+        <v>79</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>12:12:27</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>13:44</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>92</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>12:12:27</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>103</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>12:12:27</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>104</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>12:12:27</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
         <v>107</v>
       </c>
-      <c r="E117" t="inlineStr">
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>12:12:27</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>14:04</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>112</v>
+      </c>
+      <c r="E126" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3281,7 +3506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3294,14 +3519,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:44:42</t>
+          <t>Última actualización: 12:12:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -3560,7 +3785,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>06:52:02</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3570,11 +3795,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>21</v>
+        <v>113</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -3585,7 +3810,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>06:52:02</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3595,11 +3820,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>113</v>
+        <v>21</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -3735,23 +3960,48 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11:44:42</t>
+          <t>12:12:27</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>43</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>12:12:27</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
           <t>13:31</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D22" t="n">
-        <v>107</v>
-      </c>
-      <c r="E22" t="inlineStr">
+      <c r="D23" t="n">
+        <v>79</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3768,7 +4018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3781,14 +4031,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:44:42</t>
+          <t>Última actualización: 12:12:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -4166,6 +4416,56 @@
       <c r="E19" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>12:12:27</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>71</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>12:12:27</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>98</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4098
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E126"/>
+  <dimension ref="A1:E134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:12:27</t>
+          <t>Última actualización: 12:46:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 121</t>
+          <t>Total filas: 129</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -783,11 +783,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>6</v>
+        <v>79</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>79</v>
+        <v>6</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -833,7 +833,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>06:52:02</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>113</v>
+        <v>21</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>06:52:02</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>21</v>
+        <v>113</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>09:23:09</t>
+          <t>10:27:56</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>27</v>
+        <v>91</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -3148,7 +3148,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>12:12:27</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -3162,7 +3162,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>11:44:42</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3187,7 +3187,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>12:12:27</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3237,7 +3237,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,21 +3248,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>12:12:27</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>13:12</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>63</v>
+        <v>26</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,21 +3273,21 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>11:44:42</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>97</v>
+        <v>29</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,21 +3298,21 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>12:12:27</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>72</v>
+        <v>35</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>12:12:27</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>13:25</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>73</v>
+        <v>38</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3353,16 +3353,16 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>13:31</t>
+          <t>13:25</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,21 +3373,21 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>12:12:27</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>13:44</t>
+          <t>13:31</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>92</v>
+        <v>45</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>12:12:27</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:44</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>103</v>
+        <v>58</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>12:12:27</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>13:56</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>104</v>
+        <v>69</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:12:27</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>13:59</t>
+          <t>13:56</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>107</v>
+        <v>70</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3478,18 +3478,218 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>107</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>12:46:44</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
           <t>14:04</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr">
+      <c r="C127" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D126" t="n">
-        <v>112</v>
-      </c>
-      <c r="E126" t="inlineStr">
+      <c r="D127" t="n">
+        <v>78</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>12:46:44</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>88</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>12:46:44</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>88</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>12:46:44</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>89</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>12:46:44</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>90</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>12:46:44</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>98</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>12:46:44</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>108</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>12:46:44</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>118</v>
+      </c>
+      <c r="E134" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3506,7 +3706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3519,14 +3719,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:12:27</t>
+          <t>Última actualización: 12:46:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -3935,7 +4135,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>11:44:42</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3949,7 +4149,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3985,7 +4185,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12:12:27</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3999,9 +4199,34 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>79</v>
+        <v>45</v>
       </c>
       <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>12:46:44</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>108</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4018,7 +4243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4031,14 +4256,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:12:27</t>
+          <t>Última actualización: 12:46:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -4397,7 +4622,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>11:44:42</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -4411,7 +4636,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>98</v>
+        <v>36</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -4447,25 +4672,75 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>12:46:44</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>13:49</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>63</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>12:12:27</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>13:50</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D21" t="n">
+      <c r="D22" t="n">
         <v>98</v>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>12:46:44</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>14:42</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>116</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4099
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E134"/>
+  <dimension ref="A1:E140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:46:44</t>
+          <t>Última actualización: 13:11:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 129</t>
+          <t>Total filas: 135</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>06:52:02</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>21</v>
+        <v>113</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:52:02</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>113</v>
+        <v>21</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>27</v>
+        <v>91</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>09:23:09</t>
+          <t>10:27:56</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3287,7 +3287,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,7 +3298,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3337,7 +3337,7 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3387,7 +3387,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>13:44</t>
+          <t>13:36</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:44</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>13:56</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>70</v>
+        <v>44</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>12:12:27</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>13:59</t>
+          <t>13:56</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>107</v>
+        <v>45</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>12:12:27</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>13:59</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>78</v>
+        <v>107</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,21 +3523,21 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>88</v>
+        <v>53</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3562,7 +3562,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3578,16 +3578,16 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>14:15</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,12 +3598,12 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -3612,7 +3612,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>90</v>
+        <v>63</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3628,16 +3628,16 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:15</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>14:34</t>
+          <t>14:15</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>108</v>
+        <v>64</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,23 +3673,173 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>65</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>13:11:40</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>73</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>13:11:40</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>14:31</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>80</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>13:11:40</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>83</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>13:11:40</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
           <t>14:44</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr">
+      <c r="C138" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D134" t="n">
-        <v>118</v>
-      </c>
-      <c r="E134" t="inlineStr">
+      <c r="D138" t="n">
+        <v>93</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>13:11:40</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>103</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>13:11:40</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>113</v>
+      </c>
+      <c r="E140" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3706,7 +3856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3719,14 +3869,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:46:44</t>
+          <t>Última actualización: 13:11:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -4185,7 +4335,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4199,7 +4349,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -4210,7 +4360,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4224,9 +4374,59 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>108</v>
+        <v>83</v>
       </c>
       <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>13:11:40</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>103</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>13:11:40</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>113</v>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4256,7 +4456,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:46:44</t>
+          <t>Última actualización: 13:11:40</t>
         </is>
       </c>
     </row>
@@ -4622,7 +4822,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -4636,7 +4836,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -4672,7 +4872,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -4686,7 +4886,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>63</v>
+        <v>38</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -4722,7 +4922,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4736,7 +4936,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>116</v>
+        <v>91</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4100
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E140"/>
+  <dimension ref="A1:E148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:11:40</t>
+          <t>Última actualización: 13:54:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 135</t>
+          <t>Total filas: 143</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>09:23:09</t>
+          <t>10:27:56</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>27</v>
+        <v>91</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>11:44:42</t>
+          <t>11:04:59</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>11:04:59</t>
+          <t>11:44:42</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3462,7 +3462,7 @@
         </is>
       </c>
       <c r="D125" t="n">
-        <v>44</v>
+        <v>1</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3487,7 +3487,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>45</v>
+        <v>2</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3523,21 +3523,21 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>53</v>
+        <v>8</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,21 +3548,21 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>63</v>
+        <v>10</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>63</v>
+        <v>20</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,12 +3623,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>14:15</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -3637,7 +3637,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>89</v>
+        <v>63</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3673,12 +3673,12 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:15</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -3687,7 +3687,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>73</v>
+        <v>22</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,21 +3723,21 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:19</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>80</v>
+        <v>25</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>14:34</t>
+          <t>14:20</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>83</v>
+        <v>26</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,21 +3773,21 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>14:44</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>93</v>
+        <v>30</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,21 +3798,21 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>14:54</t>
+          <t>14:31</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>103</v>
+        <v>37</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,23 +3823,223 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>40</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>13:54:42</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>50</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>13:54:42</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>60</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>13:54:42</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
           <t>15:04</t>
         </is>
       </c>
-      <c r="C140" t="inlineStr">
+      <c r="C143" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D140" t="n">
-        <v>113</v>
-      </c>
-      <c r="E140" t="inlineStr">
+      <c r="D143" t="n">
+        <v>70</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>13:54:42</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>15:06</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>72</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>13:54:42</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>81</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>13:54:42</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>90</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>13:54:42</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>100</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>13:54:42</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>15:44</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>110</v>
+      </c>
+      <c r="E148" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3856,7 +4056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3869,14 +4069,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:11:40</t>
+          <t>Última actualización: 13:54:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -4360,7 +4560,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4374,7 +4574,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>83</v>
+        <v>40</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4385,7 +4585,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4399,7 +4599,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>103</v>
+        <v>60</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -4410,7 +4610,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4424,9 +4624,34 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>113</v>
+        <v>70</v>
       </c>
       <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>13:54:42</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>100</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4443,7 +4668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4456,14 +4681,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:11:40</t>
+          <t>Última actualización: 13:54:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -4922,7 +5147,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4936,11 +5161,36 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>91</v>
+        <v>48</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>13:54:42</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>15:22</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>88</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4101
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E148"/>
+  <dimension ref="A1:E160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:54:42</t>
+          <t>Última actualización: 14:20:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 143</t>
+          <t>Total filas: 155</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>06:52:02</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>113</v>
+        <v>21</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>06:52:02</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>21</v>
+        <v>113</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>27</v>
+        <v>91</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>09:23:09</t>
+          <t>10:27:56</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>11:04:59</t>
+          <t>11:44:42</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>11:44:42</t>
+          <t>11:04:59</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>20</v>
+        <v>88</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>63</v>
+        <v>20</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3683,11 +3683,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>89</v>
+        <v>64</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3773,21 +3773,21 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>14:20:20</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:21</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,21 +3798,21 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>14:20:20</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,21 +3823,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>14:20:20</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>14:34</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3848,21 +3848,21 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>14:20:20</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>14:44</t>
+          <t>14:31</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3878,16 +3878,16 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>14:54</t>
+          <t>14:34</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,21 +3898,21 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>14:20:20</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,21 +3923,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>14:20:20</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>15:06</t>
+          <t>14:44</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>72</v>
+        <v>24</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3953,16 +3953,16 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>14:54</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,21 +3973,21 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>14:20:20</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>90</v>
+        <v>35</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>14:20:20</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>15:34</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>100</v>
+        <v>41</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,23 +4023,323 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
+          <t>14:20:20</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>44</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>14:20:20</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>15:06</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>46</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
           <t>13:54:42</t>
         </is>
       </c>
-      <c r="B148" t="inlineStr">
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>15:06</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>72</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>14:20:20</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>55</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>14:20:20</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>64</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>13:54:42</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>100</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>14:20:20</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>75</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>14:20:20</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
         <is>
           <t>15:44</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr">
+      <c r="C155" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D148" t="n">
-        <v>110</v>
-      </c>
-      <c r="E148" t="inlineStr">
+      <c r="D155" t="n">
+        <v>84</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>14:20:20</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>15:51</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>91</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>14:20:20</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>15:53</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>93</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>14:20:20</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>95</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>14:20:20</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>104</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>14:20:20</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>114</v>
+      </c>
+      <c r="E160" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4056,7 +4356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4069,14 +4369,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:54:42</t>
+          <t>Última actualización: 14:20:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -4585,21 +4885,21 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>14:20:20</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>14:54</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -4615,16 +4915,16 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>14:54</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -4635,23 +4935,98 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>14:20:20</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>35</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>14:20:20</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>44</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>13:54:42</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>15:34</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D27" t="n">
+      <c r="D29" t="n">
         <v>100</v>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>14:20:20</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>75</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4668,7 +5043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4681,14 +5056,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:54:42</t>
+          <t>Última actualización: 14:20:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -5172,25 +5547,100 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>14:20:20</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>14:43</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>23</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>13:54:42</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>15:22</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="D25" t="n">
         <v>88</v>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>14:20:20</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>63</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>14:20:20</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>16:03</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>103</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4102
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E160"/>
+  <dimension ref="A1:E169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:20:20</t>
+          <t>Última actualización: 14:51:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 155</t>
+          <t>Total filas: 164</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -783,11 +783,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>79</v>
+        <v>6</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>6</v>
+        <v>79</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>06:52:02</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>21</v>
+        <v>113</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:52:02</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>113</v>
+        <v>21</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>89</v>
+        <v>64</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3683,11 +3683,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>14:20:20</t>
+          <t>14:51:15</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3987,7 +3987,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>14:20:20</t>
+          <t>14:51:15</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4012,7 +4012,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4048,21 +4048,21 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>14:20:20</t>
+          <t>14:51:15</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>15:06</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,7 +4073,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>14:51:15</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4083,11 +4083,11 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>72</v>
+        <v>15</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,21 +4098,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>14:20:20</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,21 +4123,21 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>14:20:20</t>
+          <t>14:51:15</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>64</v>
+        <v>24</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,21 +4148,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>14:51:15</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>15:34</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>100</v>
+        <v>33</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,12 +4173,12 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>14:20:20</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:34</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -4187,7 +4187,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,21 +4198,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>14:20:20</t>
+          <t>14:51:15</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>15:44</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>84</v>
+        <v>44</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,21 +4223,21 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>14:20:20</t>
+          <t>14:51:15</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>15:51</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>91</v>
+        <v>50</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4253,16 +4253,16 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>15:53</t>
+          <t>15:44</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,21 +4273,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>14:20:20</t>
+          <t>14:51:15</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>95</v>
+        <v>54</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,21 +4298,21 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>14:20:20</t>
+          <t>14:51:15</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>104</v>
+        <v>59</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4328,18 +4328,243 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
+          <t>15:51</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>91</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>14:20:20</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>15:53</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>93</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>14:51:15</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>63</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>14:51:15</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>64</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>14:51:15</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>73</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>14:51:15</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
           <t>16:14</t>
         </is>
       </c>
-      <c r="C160" t="inlineStr">
+      <c r="C165" t="inlineStr">
         <is>
           <t>17X38_ROMERO</t>
         </is>
       </c>
-      <c r="D160" t="n">
-        <v>114</v>
-      </c>
-      <c r="E160" t="inlineStr">
+      <c r="D165" t="n">
+        <v>83</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>14:51:15</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>93</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>14:51:15</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>103</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>14:51:15</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>104</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>14:51:15</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>113</v>
+      </c>
+      <c r="E169" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4356,7 +4581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4369,14 +4594,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:20:20</t>
+          <t>Última actualización: 14:51:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -4935,7 +5160,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>14:20:20</t>
+          <t>14:51:15</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4949,7 +5174,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -4985,21 +5210,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>14:51:15</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>15:34</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>100</v>
+        <v>14</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -5010,23 +5235,48 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>14:20:20</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>100</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>14:51:15</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>15:35</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D30" t="n">
-        <v>75</v>
-      </c>
-      <c r="E30" t="inlineStr">
+      <c r="D31" t="n">
+        <v>44</v>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5043,7 +5293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5056,14 +5306,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:20:20</t>
+          <t>Última actualización: 14:51:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -5597,7 +5847,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>14:20:20</t>
+          <t>14:51:15</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -5611,7 +5861,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -5622,7 +5872,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>14:20:20</t>
+          <t>14:51:15</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5636,11 +5886,36 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>103</v>
+        <v>72</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>14:51:15</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>99</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4103
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E169"/>
+  <dimension ref="A1:E175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:51:15</t>
+          <t>Última actualización: 15:21:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 164</t>
+          <t>Total filas: 170</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -833,7 +833,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3683,11 +3683,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>89</v>
+        <v>64</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -4073,7 +4073,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>14:51:15</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4083,11 +4083,11 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>15</v>
+        <v>72</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,7 +4098,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>14:51:15</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -4108,11 +4108,11 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>72</v>
+        <v>15</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>14:51:15</t>
+          <t>15:21:43</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4162,7 +4162,7 @@
         </is>
       </c>
       <c r="D153" t="n">
-        <v>33</v>
+        <v>3</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,7 +4173,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>15:21:43</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4187,7 +4187,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>100</v>
+        <v>13</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4223,7 +4223,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>14:51:15</t>
+          <t>15:21:43</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,7 +4248,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>14:20:20</t>
+          <t>15:21:43</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -4262,7 +4262,7 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>84</v>
+        <v>23</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>14:20:20</t>
+          <t>15:21:43</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4337,7 +4337,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>91</v>
+        <v>30</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4398,7 +4398,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>14:51:15</t>
+          <t>15:21:43</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4412,7 +4412,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>14:51:15</t>
+          <t>15:21:43</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>73</v>
+        <v>35</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>14:51:15</t>
+          <t>15:21:43</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>83</v>
+        <v>43</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,21 +4473,21 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>14:51:15</t>
+          <t>15:21:43</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:14</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>93</v>
+        <v>53</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,21 +4498,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>14:51:15</t>
+          <t>15:21:43</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:16</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>103</v>
+        <v>55</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,21 +4523,21 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>14:51:15</t>
+          <t>15:21:43</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:24</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>104</v>
+        <v>63</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,23 +4548,173 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>14:51:15</t>
+          <t>15:21:43</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>73</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>15:21:43</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>74</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>15:21:43</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>80</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>15:21:43</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
           <t>16:44</t>
         </is>
       </c>
-      <c r="C169" t="inlineStr">
+      <c r="C172" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D169" t="n">
+      <c r="D172" t="n">
+        <v>83</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>15:21:43</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>94</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>15:21:43</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>17:04</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>103</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>15:21:43</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>17:14</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
         <v>113</v>
       </c>
-      <c r="E169" t="inlineStr">
+      <c r="E175" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4581,7 +4731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4594,14 +4744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:51:15</t>
+          <t>Última actualización: 15:21:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 27</t>
         </is>
       </c>
     </row>
@@ -5235,7 +5385,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>15:21:43</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5249,7 +5399,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>100</v>
+        <v>13</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -5277,6 +5427,31 @@
         <v>44</v>
       </c>
       <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>15:21:43</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>17:14</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>113</v>
+      </c>
+      <c r="E32" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5293,7 +5468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5306,14 +5481,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:51:15</t>
+          <t>Última actualización: 15:21:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -5822,7 +5997,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>15:21:43</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -5836,7 +6011,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>88</v>
+        <v>1</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -5872,12 +6047,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>14:51:15</t>
+          <t>15:21:43</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>16:03</t>
+          <t>16:02</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -5886,7 +6061,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>72</v>
+        <v>41</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -5902,18 +6077,68 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
+          <t>16:03</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>72</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>15:21:43</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>16:29</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>68</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>14:51:15</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>16:30</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D28" t="n">
+      <c r="D30" t="n">
         <v>99</v>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4104
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E175"/>
+  <dimension ref="A1:E183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:21:43</t>
+          <t>Última actualización: 16:08:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 170</t>
+          <t>Total filas: 178</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>09:23:09</t>
+          <t>10:27:56</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>27</v>
+        <v>91</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>11:44:42</t>
+          <t>11:04:59</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>11:04:59</t>
+          <t>11:44:42</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -4473,7 +4473,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>15:21:43</t>
+          <t>16:08:49</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4487,7 +4487,7 @@
         </is>
       </c>
       <c r="D166" t="n">
-        <v>53</v>
+        <v>6</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>15:21:43</t>
+          <t>16:08:49</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4512,7 +4512,7 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>55</v>
+        <v>8</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,7 +4523,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>15:21:43</t>
+          <t>16:08:49</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -4537,7 +4537,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>63</v>
+        <v>16</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,7 +4548,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>15:21:43</t>
+          <t>16:08:49</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -4562,7 +4562,7 @@
         </is>
       </c>
       <c r="D169" t="n">
-        <v>73</v>
+        <v>26</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>15:21:43</t>
+          <t>16:08:49</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -4587,7 +4587,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>74</v>
+        <v>27</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>15:21:43</t>
+          <t>16:08:49</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4612,7 +4612,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>15:21:43</t>
+          <t>16:08:49</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>83</v>
+        <v>36</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>15:21:43</t>
+          <t>16:08:49</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:51</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>94</v>
+        <v>43</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>15:21:43</t>
+          <t>16:08:49</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>103</v>
+        <v>47</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,23 +4698,223 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>15:21:43</t>
+          <t>16:08:49</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
+          <t>17:04</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>56</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>16:08:49</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
           <t>17:14</t>
         </is>
       </c>
-      <c r="C175" t="inlineStr">
+      <c r="C176" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D175" t="n">
-        <v>113</v>
-      </c>
-      <c r="E175" t="inlineStr">
+      <c r="D176" t="n">
+        <v>66</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>16:08:49</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>76</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>16:08:49</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>17:34</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>86</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>16:08:49</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>17:34</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>86</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>16:08:49</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>87</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>16:08:49</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>17:44</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>96</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>16:08:49</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>17:54</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>106</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>16:08:49</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>107</v>
+      </c>
+      <c r="E183" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4731,7 +4931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4744,14 +4944,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:21:43</t>
+          <t>Última actualización: 16:08:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 27</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -5435,7 +5635,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>15:21:43</t>
+          <t>16:08:49</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5449,9 +5649,59 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>113</v>
+        <v>66</v>
       </c>
       <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>16:08:49</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>17:44</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>96</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>16:08:49</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>17:54</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>106</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5468,7 +5718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5481,14 +5731,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:21:43</t>
+          <t>Última actualización: 16:08:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -6097,7 +6347,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>15:21:43</t>
+          <t>16:08:49</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -6111,7 +6361,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>68</v>
+        <v>21</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -6141,6 +6391,31 @@
       <c r="E30" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>16:08:49</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>74</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4105
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E183"/>
+  <dimension ref="A1:E191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:08:49</t>
+          <t>Última actualización: 16:44:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 178</t>
+          <t>Total filas: 186</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -783,11 +783,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>6</v>
+        <v>79</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>79</v>
+        <v>6</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>27</v>
+        <v>91</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>09:23:09</t>
+          <t>10:27:56</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>11:04:59</t>
+          <t>11:44:42</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>11:44:42</t>
+          <t>11:04:59</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>88</v>
+        <v>20</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>20</v>
+        <v>63</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>89</v>
+        <v>64</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3683,11 +3683,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>16:08:49</t>
+          <t>16:44:41</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>16:08:49</t>
+          <t>16:44:41</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>16:51</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>43</v>
+        <v>1</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>16:08:49</t>
+          <t>16:44:41</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:51</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>47</v>
+        <v>7</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,21 +4698,21 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>16:08:49</t>
+          <t>16:44:41</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>56</v>
+        <v>11</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,21 +4723,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>16:08:49</t>
+          <t>16:44:41</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>17:14</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>66</v>
+        <v>20</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,21 +4748,21 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>16:08:49</t>
+          <t>16:44:41</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>76</v>
+        <v>30</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>16:08:49</t>
+          <t>16:44:41</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>17:34</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>86</v>
+        <v>40</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>16:08:49</t>
+          <t>16:44:41</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>17:34</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>86</v>
+        <v>47</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4828,16 +4828,16 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:34</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4853,16 +4853,16 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>17:44</t>
+          <t>17:34</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>16:08:49</t>
+          <t>16:44:41</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>17:54</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>106</v>
+        <v>51</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,23 +4898,223 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
+          <t>16:44:41</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>52</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>16:44:41</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>17:44</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>60</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>16:44:41</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>17:54</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>70</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
           <t>16:08:49</t>
         </is>
       </c>
-      <c r="B183" t="inlineStr">
+      <c r="B186" t="inlineStr">
         <is>
           <t>17:55</t>
         </is>
       </c>
-      <c r="C183" t="inlineStr">
+      <c r="C186" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D183" t="n">
+      <c r="D186" t="n">
         <v>107</v>
       </c>
-      <c r="E183" t="inlineStr">
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>16:44:41</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>18:04</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>80</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>16:44:41</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>18:14</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>90</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>16:44:41</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>100</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>16:44:41</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>18:34</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>110</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>16:44:41</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>112</v>
+      </c>
+      <c r="E191" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4931,7 +5131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4944,14 +5144,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:08:49</t>
+          <t>Última actualización: 16:44:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -5635,7 +5835,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>16:08:49</t>
+          <t>16:44:41</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5649,7 +5849,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>66</v>
+        <v>30</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5660,7 +5860,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>16:08:49</t>
+          <t>16:44:41</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -5674,7 +5874,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>96</v>
+        <v>60</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -5685,7 +5885,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>16:08:49</t>
+          <t>16:44:41</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -5699,9 +5899,34 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>106</v>
+        <v>70</v>
       </c>
       <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>16:44:41</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>18:14</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>90</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5731,7 +5956,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:08:49</t>
+          <t>Última actualización: 16:44:41</t>
         </is>
       </c>
     </row>
@@ -6397,7 +6622,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>16:08:49</t>
+          <t>16:44:41</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -6411,7 +6636,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>74</v>
+        <v>38</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4106
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E191"/>
+  <dimension ref="A1:E203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:44:41</t>
+          <t>Última actualización: 17:04:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 186</t>
+          <t>Total filas: 198</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>09:23:09</t>
+          <t>10:27:56</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>27</v>
+        <v>91</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -4073,7 +4073,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>14:51:15</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4083,11 +4083,11 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>72</v>
+        <v>15</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,7 +4098,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>14:51:15</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -4108,11 +4108,11 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>15</v>
+        <v>72</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4748,21 +4748,21 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>16:44:41</t>
+          <t>17:04:13</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>17:14</t>
+          <t>17:06</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4778,16 +4778,16 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>16:44:41</t>
+          <t>17:04:13</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>17:31</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>47</v>
+        <v>11</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,21 +4823,21 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>16:08:49</t>
+          <t>17:04:13</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>17:34</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>86</v>
+        <v>20</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,21 +4848,21 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>16:08:49</t>
+          <t>17:04:13</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>17:34</t>
+          <t>17:26</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>86</v>
+        <v>22</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>16:44:41</t>
+          <t>17:04:13</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,21 +4898,21 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>16:44:41</t>
+          <t>16:08:49</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:34</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,21 +4923,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>16:44:41</t>
+          <t>16:08:49</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>17:44</t>
+          <t>17:34</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>16:44:41</t>
+          <t>17:04:13</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>17:54</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>70</v>
+        <v>31</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>16:08:49</t>
+          <t>16:44:41</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>107</v>
+        <v>52</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,21 +4998,21 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>16:44:41</t>
+          <t>17:04:13</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>18:04</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5028,16 +5028,16 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>18:14</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>16:44:41</t>
+          <t>17:04:13</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>100</v>
+        <v>41</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5078,16 +5078,16 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>17:54</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>110</v>
+        <v>70</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,23 +5098,323 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
+          <t>17:04:13</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>51</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>16:08:49</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>107</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>17:04:13</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>18:04</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>60</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
           <t>16:44:41</t>
         </is>
       </c>
-      <c r="B191" t="inlineStr">
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>18:14</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>90</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>17:04:13</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>71</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>16:44:41</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>100</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>17:04:13</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>81</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>17:04:13</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>18:31</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>87</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>17:04:13</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>18:34</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>90</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>17:04:13</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
         <is>
           <t>18:36</t>
         </is>
       </c>
-      <c r="C191" t="inlineStr">
+      <c r="C200" t="inlineStr">
         <is>
           <t>16_SANTA ANA</t>
         </is>
       </c>
-      <c r="D191" t="n">
-        <v>112</v>
-      </c>
-      <c r="E191" t="inlineStr">
+      <c r="D200" t="n">
+        <v>92</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>17:04:13</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>100</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>17:04:13</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>18:54</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>110</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>17:04:13</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>116</v>
+      </c>
+      <c r="E203" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5131,7 +5431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5144,14 +5444,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:44:41</t>
+          <t>Última actualización: 17:04:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -5860,21 +6160,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>16:44:41</t>
+          <t>17:04:13</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>17:44</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>60</v>
+        <v>11</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -5890,16 +6190,16 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>17:54</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -5910,23 +6210,148 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>17:04:13</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>41</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>16:44:41</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>17:54</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>70</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>17:04:13</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>51</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>16:44:41</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
         <is>
           <t>18:14</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D35" t="n">
+      <c r="D38" t="n">
         <v>90</v>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>17:04:13</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>71</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>17:04:13</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>116</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5943,7 +6368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5956,14 +6381,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:44:41</t>
+          <t>Última actualización: 17:04:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -6639,6 +7064,56 @@
         <v>38</v>
       </c>
       <c r="E31" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>17:04:13</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>17:23</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>19</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>17:04:13</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>101</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4107
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E203"/>
+  <dimension ref="A1:E210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:04:13</t>
+          <t>Última actualización: 17:46:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 198</t>
+          <t>Total filas: 205</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -783,11 +783,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>79</v>
+        <v>6</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>6</v>
+        <v>79</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -833,7 +833,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>27</v>
+        <v>91</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>09:23:09</t>
+          <t>10:27:56</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>20</v>
+        <v>88</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>63</v>
+        <v>20</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -4908,7 +4908,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -4933,7 +4933,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>17:04:13</t>
+          <t>17:46:10</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5112,7 +5112,7 @@
         </is>
       </c>
       <c r="D191" t="n">
-        <v>51</v>
+        <v>9</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>17:04:13</t>
+          <t>17:46:10</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5162,7 +5162,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5198,7 +5198,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>17:04:13</t>
+          <t>17:46:10</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -5212,7 +5212,7 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,21 +5223,21 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>16:44:41</t>
+          <t>17:46:10</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>100</v>
+        <v>35</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,12 +5248,12 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>17:04:13</t>
+          <t>16:44:41</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -5262,7 +5262,7 @@
         </is>
       </c>
       <c r="D197" t="n">
-        <v>81</v>
+        <v>100</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,21 +5273,21 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>17:04:13</t>
+          <t>17:46:10</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>18:31</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>87</v>
+        <v>39</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5303,16 +5303,16 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:31</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,21 +5323,21 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>17:04:13</t>
+          <t>17:46:10</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>92</v>
+        <v>48</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,21 +5348,21 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>17:04:13</t>
+          <t>17:46:10</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>18:44</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>17:04:13</t>
+          <t>17:46:10</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>18:54</t>
+          <t>18:44</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>110</v>
+        <v>58</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,23 +5398,198 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>17:04:13</t>
+          <t>17:46:10</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
+          <t>18:54</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>68</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>17:46:10</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="C203" t="inlineStr">
+      <c r="C204" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D203" t="n">
-        <v>116</v>
-      </c>
-      <c r="E203" t="inlineStr">
+      <c r="D204" t="n">
+        <v>74</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>17:46:10</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>79</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>17:46:10</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>19:14</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>88</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>17:46:10</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>90</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>17:46:10</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>91</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>17:46:10</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>98</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>17:46:10</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>99</v>
+      </c>
+      <c r="E210" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5431,7 +5606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5444,14 +5619,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:04:13</t>
+          <t>Última actualización: 17:46:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -6260,7 +6435,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>17:04:13</t>
+          <t>17:46:10</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6274,7 +6449,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>51</v>
+        <v>9</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -6310,7 +6485,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>17:04:13</t>
+          <t>17:46:10</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -6324,7 +6499,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -6335,7 +6510,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>17:04:13</t>
+          <t>17:46:10</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -6349,9 +6524,34 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>116</v>
+        <v>74</v>
       </c>
       <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>17:46:10</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>99</v>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6368,7 +6568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6381,14 +6581,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:04:13</t>
+          <t>Última actualización: 17:46:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -7097,7 +7297,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>17:04:13</t>
+          <t>17:46:10</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -7111,11 +7311,36 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>101</v>
+        <v>59</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>17:46:10</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>89</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4108
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E210"/>
+  <dimension ref="A1:E217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:46:10</t>
+          <t>Última actualización: 18:13:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 205</t>
+          <t>Total filas: 212</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -783,11 +783,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>6</v>
+        <v>79</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>79</v>
+        <v>6</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -833,7 +833,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>06:52:02</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>113</v>
+        <v>21</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>06:52:02</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>21</v>
+        <v>113</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3683,11 +3683,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>89</v>
+        <v>64</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -4073,7 +4073,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>14:51:15</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4083,11 +4083,11 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>15</v>
+        <v>72</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,7 +4098,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>14:51:15</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -4108,11 +4108,11 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>72</v>
+        <v>15</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>17:46:10</t>
+          <t>16:08:49</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5108,11 +5108,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>9</v>
+        <v>107</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>16:08:49</t>
+          <t>17:46:10</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>107</v>
+        <v>9</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>16:44:41</t>
+          <t>18:13:42</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5187,7 +5187,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>90</v>
+        <v>1</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>17:46:10</t>
+          <t>18:13:42</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5237,7 +5237,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>16:44:41</t>
+          <t>18:13:42</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5262,7 +5262,7 @@
         </is>
       </c>
       <c r="D197" t="n">
-        <v>100</v>
+        <v>11</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>17:46:10</t>
+          <t>18:13:42</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5337,7 +5337,7 @@
         </is>
       </c>
       <c r="D200" t="n">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>17:46:10</t>
+          <t>18:13:42</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5362,7 +5362,7 @@
         </is>
       </c>
       <c r="D201" t="n">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>17:46:10</t>
+          <t>18:13:42</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5387,7 +5387,7 @@
         </is>
       </c>
       <c r="D202" t="n">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>17:46:10</t>
+          <t>18:13:42</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5412,7 +5412,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>68</v>
+        <v>41</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,12 +5423,12 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>17:46:10</t>
+          <t>18:13:42</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:59</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -5437,7 +5437,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>74</v>
+        <v>46</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5453,16 +5453,16 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,21 +5473,21 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>17:46:10</t>
+          <t>18:13:42</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>19:14</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>88</v>
+        <v>51</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5503,16 +5503,16 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5528,16 +5528,16 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:14</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>17:46:10</t>
+          <t>18:13:42</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>98</v>
+        <v>63</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,23 +5573,198 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
+          <t>18:13:42</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>63</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
           <t>17:46:10</t>
         </is>
       </c>
-      <c r="B210" t="inlineStr">
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>91</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>18:13:42</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>19:21</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>68</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>18:13:42</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>71</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>18:13:42</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>71</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>17:46:10</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
         <is>
           <t>19:25</t>
         </is>
       </c>
-      <c r="C210" t="inlineStr">
+      <c r="C215" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D210" t="n">
+      <c r="D215" t="n">
         <v>99</v>
       </c>
-      <c r="E210" t="inlineStr">
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>18:13:42</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>96</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>18:13:42</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>97</v>
+      </c>
+      <c r="E217" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5606,7 +5781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5619,14 +5794,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:46:10</t>
+          <t>Última actualización: 18:13:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 36</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -5835,7 +6010,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -5845,11 +6020,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -5860,7 +6035,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -5870,11 +6045,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -5885,7 +6060,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>06:52:02</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -5895,11 +6070,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>113</v>
+        <v>21</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -5910,7 +6085,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>06:52:02</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -5920,11 +6095,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>21</v>
+        <v>113</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -6460,7 +6635,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>16:44:41</t>
+          <t>18:13:42</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -6474,7 +6649,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>90</v>
+        <v>1</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -6510,12 +6685,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>17:46:10</t>
+          <t>18:13:42</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:59</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -6524,7 +6699,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>74</v>
+        <v>46</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -6540,18 +6715,68 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>74</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>18:13:42</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>71</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>17:46:10</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>19:25</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D41" t="n">
+      <c r="D43" t="n">
         <v>99</v>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6568,7 +6793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6581,14 +6806,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:46:10</t>
+          <t>Última actualización: 18:13:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -7297,12 +7522,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>17:46:10</t>
+          <t>18:13:42</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>18:45</t>
+          <t>18:44</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -7311,7 +7536,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -7327,20 +7552,95 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>59</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>18:13:42</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>19:14</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>61</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>17:46:10</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>19:15</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D34" t="n">
+      <c r="D36" t="n">
         <v>89</v>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>18:13:42</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>19:46</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>93</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4109
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E217"/>
+  <dimension ref="A1:E224"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:13:42</t>
+          <t>Última actualización: 18:48:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 212</t>
+          <t>Total filas: 219</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>06:52:02</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>21</v>
+        <v>113</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:52:02</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>113</v>
+        <v>21</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>09:23:09</t>
+          <t>10:27:56</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>27</v>
+        <v>91</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>89</v>
+        <v>64</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3683,11 +3683,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -4908,7 +4908,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -4933,7 +4933,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>18:13:42</t>
+          <t>18:48:20</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5412,7 +5412,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>41</v>
+        <v>6</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5448,7 +5448,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>17:46:10</t>
+          <t>18:48:20</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -5462,7 +5462,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>74</v>
+        <v>12</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,7 +5473,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>18:13:42</t>
+          <t>18:48:20</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5487,7 +5487,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>51</v>
+        <v>16</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5523,12 +5523,12 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>17:46:10</t>
+          <t>18:48:20</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>19:14</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -5537,7 +5537,7 @@
         </is>
       </c>
       <c r="D208" t="n">
-        <v>88</v>
+        <v>23</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>18:13:42</t>
+          <t>17:46:10</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:14</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>17:46:10</t>
+          <t>18:48:20</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>91</v>
+        <v>28</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,21 +5623,21 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>18:13:42</t>
+          <t>18:48:20</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>68</v>
+        <v>29</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5653,16 +5653,16 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5698,21 +5698,21 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>17:46:10</t>
+          <t>18:48:20</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>99</v>
+        <v>36</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,21 +5723,21 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>18:13:42</t>
+          <t>18:48:20</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>96</v>
+        <v>37</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,23 +5748,198 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>18:13:42</t>
+          <t>18:48:20</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>61</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>18:48:20</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
           <t>19:50</t>
         </is>
       </c>
-      <c r="C217" t="inlineStr">
+      <c r="C218" t="inlineStr">
         <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D217" t="n">
-        <v>97</v>
-      </c>
-      <c r="E217" t="inlineStr">
+      <c r="D218" t="n">
+        <v>62</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>18:48:20</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>19:56</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>68</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>18:48:20</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>73</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>18:48:20</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>87</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>18:48:20</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>87</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>18:48:20</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>111</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>18:48:20</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>113</v>
+      </c>
+      <c r="E224" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5781,7 +5956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5794,14 +5969,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:13:42</t>
+          <t>Última actualización: 18:48:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 41</t>
         </is>
       </c>
     </row>
@@ -6010,7 +6185,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -6020,11 +6195,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -6035,7 +6210,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -6045,11 +6220,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -6710,7 +6885,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>17:46:10</t>
+          <t>18:48:20</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -6724,7 +6899,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>74</v>
+        <v>12</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -6760,7 +6935,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>17:46:10</t>
+          <t>18:48:20</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -6774,9 +6949,84 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>99</v>
+        <v>37</v>
       </c>
       <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>18:48:20</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>87</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>18:48:20</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>111</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>18:48:20</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>113</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6793,7 +7043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6806,14 +7056,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:13:42</t>
+          <t>Última actualización: 18:48:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -7572,37 +7822,37 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>18:13:42</t>
+          <t>18:48:20</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>19:14</t>
+          <t>18:48</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>17:46:10</t>
+          <t>18:13:42</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>19:15</t>
+          <t>19:14</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -7611,7 +7861,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>89</v>
+        <v>61</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -7622,23 +7872,73 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>18:48:20</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>27</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>18:13:42</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>19:46</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D37" t="n">
+      <c r="D38" t="n">
         <v>93</v>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>18:48:20</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>59</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4110
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E224"/>
+  <dimension ref="A1:E231"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:48:20</t>
+          <t>Última actualización: 19:12:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 219</t>
+          <t>Total filas: 226</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -773,7 +773,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -783,11 +783,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>79</v>
+        <v>6</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>6</v>
+        <v>79</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -833,7 +833,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3683,11 +3683,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>89</v>
+        <v>64</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -5548,12 +5548,12 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>17:46:10</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>19:14</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -5562,7 +5562,7 @@
         </is>
       </c>
       <c r="D209" t="n">
-        <v>88</v>
+        <v>0</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,21 +5573,21 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>18:13:42</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>18:48:20</t>
+          <t>17:46:10</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:14</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>28</v>
+        <v>88</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,12 +5623,12 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>18:48:20</t>
+          <t>18:13:42</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -5637,7 +5637,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>29</v>
+        <v>63</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>18:13:42</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,21 +5673,21 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>18:13:42</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>71</v>
+        <v>5</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,21 +5698,21 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>18:48:20</t>
+          <t>18:13:42</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>36</v>
+        <v>68</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,21 +5723,21 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>18:48:20</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,21 +5748,21 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>18:48:20</t>
+          <t>18:13:42</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,21 +5773,21 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>18:48:20</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>19:50</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>62</v>
+        <v>13</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,21 +5798,21 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>18:48:20</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>19:56</t>
+          <t>19:49</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>68</v>
+        <v>37</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,21 +5823,21 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>18:48:20</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:50</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>73</v>
+        <v>38</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,21 +5848,21 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>18:48:20</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>19:56</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>87</v>
+        <v>44</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,21 +5873,21 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>18:48:20</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>87</v>
+        <v>49</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,21 +5898,21 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>18:48:20</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>111</v>
+        <v>63</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5928,18 +5928,193 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>87</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>19:12:14</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>20:16</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>64</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>18:48:20</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>111</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>19:12:14</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>88</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>19:12:14</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
           <t>20:41</t>
         </is>
       </c>
-      <c r="C224" t="inlineStr">
+      <c r="C228" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D224" t="n">
-        <v>113</v>
-      </c>
-      <c r="E224" t="inlineStr">
+      <c r="D228" t="n">
+        <v>89</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>19:12:14</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>105</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>19:12:14</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>114</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>19:12:14</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>114</v>
+      </c>
+      <c r="E231" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5956,7 +6131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5969,14 +6144,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:48:20</t>
+          <t>Última actualización: 19:12:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 41</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -6235,7 +6410,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>06:52:02</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -6245,11 +6420,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>21</v>
+        <v>113</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -6260,7 +6435,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>06:52:02</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -6270,11 +6445,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>113</v>
+        <v>21</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -6935,7 +7110,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>18:48:20</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -6949,7 +7124,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -6960,7 +7135,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>18:48:20</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -6974,7 +7149,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>87</v>
+        <v>63</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -7010,23 +7185,73 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>18:48:20</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>88</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>19:12:14</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
           <t>20:41</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D46" t="n">
-        <v>113</v>
-      </c>
-      <c r="E46" t="inlineStr">
+      <c r="D47" t="n">
+        <v>89</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>19:12:14</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>114</v>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7043,7 +7268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7056,14 +7281,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:48:20</t>
+          <t>Última actualización: 19:12:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 34</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -7872,7 +8097,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>18:48:20</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7886,7 +8111,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -7922,7 +8147,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>18:48:20</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -7936,9 +8161,34 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>59</v>
+        <v>35</v>
       </c>
       <c r="E39" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>19:12:14</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>87</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4111
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E231"/>
+  <dimension ref="A1:E240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:12:14</t>
+          <t>Última actualización: 19:49:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 226</t>
+          <t>Total filas: 235</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -833,7 +833,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>27</v>
+        <v>91</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>09:23:09</t>
+          <t>10:27:56</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>11:44:42</t>
+          <t>11:04:59</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>11:04:59</t>
+          <t>11:44:42</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>89</v>
+        <v>64</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3683,11 +3683,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -4908,7 +4908,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -4933,7 +4933,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>18:13:42</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>12</v>
+        <v>71</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>18:13:42</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>71</v>
+        <v>12</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5798,7 +5798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>19:49:52</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5812,7 +5812,7 @@
         </is>
       </c>
       <c r="D219" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,7 +5823,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>19:49:52</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -5833,11 +5833,11 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5853,16 +5853,16 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>19:56</t>
+          <t>19:50</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,21 +5873,21 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>19:49:52</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:51</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>49</v>
+        <v>2</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,21 +5898,21 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>19:49:52</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>19:56</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>63</v>
+        <v>7</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,21 +5923,21 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>18:48:20</t>
+          <t>19:49:52</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>87</v>
+        <v>12</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,21 +5948,21 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>19:49:52</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>64</v>
+        <v>25</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,21 +5973,21 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>18:48:20</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>111</v>
+        <v>63</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>19:49:52</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>88</v>
+        <v>26</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6028,16 +6028,16 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:16</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>89</v>
+        <v>64</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,21 +6048,21 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>19:49:52</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6078,16 +6078,16 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>20:40</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>114</v>
+        <v>88</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,23 +6098,248 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
+          <t>19:49:52</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>52</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>19:49:52</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>20:54</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>65</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>19:49:52</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>67</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
           <t>19:12:14</t>
         </is>
       </c>
-      <c r="B231" t="inlineStr">
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>105</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>19:49:52</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>21:05</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>76</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>19:49:52</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
         <is>
           <t>21:06</t>
         </is>
       </c>
-      <c r="C231" t="inlineStr">
+      <c r="C236" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D231" t="n">
+      <c r="D236" t="n">
+        <v>77</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>19:12:14</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
         <v>114</v>
       </c>
-      <c r="E231" t="inlineStr">
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>19:49:52</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>21:12</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>83</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>19:49:52</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>105</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>19:49:52</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>107</v>
+      </c>
+      <c r="E240" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6131,7 +6356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6144,14 +6369,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:12:14</t>
+          <t>Última actualización: 19:49:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 43</t>
+          <t>Total filas: 44</t>
         </is>
       </c>
     </row>
@@ -7135,12 +7360,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>19:49:52</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -7149,7 +7374,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>63</v>
+        <v>25</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -7160,21 +7385,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>18:48:20</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>111</v>
+        <v>63</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -7185,12 +7410,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>19:49:52</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -7199,7 +7424,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>88</v>
+        <v>50</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -7215,16 +7440,16 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:40</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -7235,23 +7460,48 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>19:49:52</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>52</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>19:49:52</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
           <t>21:06</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D48" t="n">
-        <v>114</v>
-      </c>
-      <c r="E48" t="inlineStr">
+      <c r="D49" t="n">
+        <v>77</v>
+      </c>
+      <c r="E49" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7268,7 +7518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7281,14 +7531,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:12:14</t>
+          <t>Última actualización: 19:49:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -8172,7 +8422,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>19:49:52</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -8186,9 +8436,34 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>87</v>
+        <v>50</v>
       </c>
       <c r="E40" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>19:49:52</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>21:31</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>102</v>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4112
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E240"/>
+  <dimension ref="A1:E247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:49:52</t>
+          <t>Última actualización: 20:13:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 235</t>
+          <t>Total filas: 242</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3683,11 +3683,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>89</v>
+        <v>64</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>18:13:42</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>71</v>
+        <v>12</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>18:13:42</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>12</v>
+        <v>71</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5823,7 +5823,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>19:49:52</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -5833,11 +5833,11 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,7 +5848,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>19:49:52</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -5858,11 +5858,11 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5948,21 +5948,21 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>19:49:52</t>
+          <t>20:13:25</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>20:13</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,12 +5973,12 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>19:49:52</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -5987,7 +5987,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>63</v>
+        <v>25</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>19:49:52</t>
+          <t>20:13:25</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6008,11 +6008,11 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,12 +6023,12 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>20:13:25</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -6037,7 +6037,7 @@
         </is>
       </c>
       <c r="D228" t="n">
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,21 +6048,21 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>19:49:52</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:16</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,12 +6073,12 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>20:13:25</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -6087,7 +6087,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>88</v>
+        <v>26</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,21 +6098,21 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>19:49:52</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:40</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>52</v>
+        <v>88</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>19:49:52</t>
+          <t>20:13:25</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>20:54</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>65</v>
+        <v>28</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>19:49:52</t>
+          <t>20:13:25</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,21 +6173,21 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>19:49:52</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:54</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>105</v>
+        <v>65</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,21 +6198,21 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>19:49:52</t>
+          <t>20:13:25</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>21:05</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>76</v>
+        <v>43</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,21 +6223,21 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>19:49:52</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>77</v>
+        <v>105</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6248,12 +6248,12 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>19:49:52</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>21:05</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -6262,7 +6262,7 @@
         </is>
       </c>
       <c r="D237" t="n">
-        <v>114</v>
+        <v>76</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6273,21 +6273,21 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>19:49:52</t>
+          <t>20:13:25</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>21:12</t>
+          <t>21:06</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>83</v>
+        <v>53</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,21 +6298,21 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>19:49:52</t>
+          <t>20:13:25</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:06</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>105</v>
+        <v>53</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6328,18 +6328,193 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
+          <t>21:12</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>83</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>20:13:25</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>81</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>20:13:25</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>82</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>19:49:52</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
           <t>21:36</t>
         </is>
       </c>
-      <c r="C240" t="inlineStr">
+      <c r="C243" t="inlineStr">
         <is>
           <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
-      <c r="D240" t="n">
+      <c r="D243" t="n">
         <v>107</v>
       </c>
-      <c r="E240" t="inlineStr">
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>20:13:25</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>83</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>20:13:25</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>84</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>20:13:25</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>21:42</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>89</v>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>20:13:25</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>21:59</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>106</v>
+      </c>
+      <c r="E247" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6369,7 +6544,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:49:52</t>
+          <t>Última actualización: 20:13:25</t>
         </is>
       </c>
     </row>
@@ -7385,7 +7560,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>20:13:25</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -7399,7 +7574,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>63</v>
+        <v>2</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -7410,7 +7585,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>19:49:52</t>
+          <t>20:13:25</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -7424,7 +7599,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -7460,7 +7635,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>19:49:52</t>
+          <t>20:13:25</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -7474,7 +7649,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -7485,7 +7660,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>19:49:52</t>
+          <t>20:13:25</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -7499,7 +7674,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>77</v>
+        <v>53</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -7518,7 +7693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7531,14 +7706,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:49:52</t>
+          <t>Última actualización: 20:13:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 36</t>
+          <t>Total filas: 39</t>
         </is>
       </c>
     </row>
@@ -8447,25 +8622,100 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>20:13:25</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>20:47</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>34</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>19:49:52</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>21:31</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D41" t="n">
+      <c r="D42" t="n">
         <v>102</v>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>20:13:25</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>21:32</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>79</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>20:13:25</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>22:09</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>116</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4113
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E247"/>
+  <dimension ref="A1:E253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:13:25</t>
+          <t>Última actualización: 20:47:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 242</t>
+          <t>Total filas: 248</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -833,7 +833,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D209" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>18:13:42</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>12</v>
+        <v>71</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>18:13:42</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>71</v>
+        <v>12</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -6173,12 +6173,12 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>19:49:52</t>
+          <t>20:47:06</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>20:54</t>
+          <t>20:52</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -6187,7 +6187,7 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>65</v>
+        <v>5</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,21 +6198,21 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>20:13:25</t>
+          <t>19:49:52</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:54</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>43</v>
+        <v>65</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,12 +6223,12 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>20:13:25</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -6237,7 +6237,7 @@
         </is>
       </c>
       <c r="D236" t="n">
-        <v>105</v>
+        <v>43</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6248,21 +6248,21 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>19:49:52</t>
+          <t>20:47:06</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>21:05</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>76</v>
+        <v>10</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6273,21 +6273,21 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>20:13:25</t>
+          <t>19:49:52</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>21:05</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,7 +6298,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>20:13:25</t>
+          <t>20:47:06</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -6308,11 +6308,11 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>53</v>
+        <v>19</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,21 +6323,21 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>19:49:52</t>
+          <t>20:47:06</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>21:12</t>
+          <t>21:06</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>83</v>
+        <v>19</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6348,21 +6348,21 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>20:13:25</t>
+          <t>19:49:52</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:12</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,21 +6373,21 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>20:13:25</t>
+          <t>20:47:06</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>21:35</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>82</v>
+        <v>47</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6398,21 +6398,21 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>19:49:52</t>
+          <t>20:13:25</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>21:35</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>107</v>
+        <v>82</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6423,7 +6423,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>20:13:25</t>
+          <t>19:49:52</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -6433,11 +6433,11 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>83</v>
+        <v>107</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,21 +6448,21 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>20:13:25</t>
+          <t>20:47:06</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>21:37</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>84</v>
+        <v>49</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,21 +6473,21 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>20:13:25</t>
+          <t>20:47:06</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>21:42</t>
+          <t>21:37</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>89</v>
+        <v>50</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6503,18 +6503,168 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
+          <t>21:42</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>89</v>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>20:47:06</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>21:50</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D248" t="n">
+        <v>63</v>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>20:47:06</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
           <t>21:59</t>
         </is>
       </c>
-      <c r="C247" t="inlineStr">
+      <c r="C249" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D247" t="n">
-        <v>106</v>
-      </c>
-      <c r="E247" t="inlineStr">
+      <c r="D249" t="n">
+        <v>72</v>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>20:47:06</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>22:07</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>80</v>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>20:47:06</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>99</v>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>20:47:06</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D252" t="n">
+        <v>110</v>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>20:47:06</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>22:41</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>114</v>
+      </c>
+      <c r="E253" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6531,7 +6681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6544,14 +6694,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:13:25</t>
+          <t>Última actualización: 20:47:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 44</t>
+          <t>Total filas: 45</t>
         </is>
       </c>
     </row>
@@ -7660,7 +7810,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>20:13:25</t>
+          <t>20:47:06</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -7674,9 +7824,34 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>53</v>
+        <v>19</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>20:47:06</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>110</v>
+      </c>
+      <c r="E50" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7706,7 +7881,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:13:25</t>
+          <t>Última actualización: 20:47:06</t>
         </is>
       </c>
     </row>
@@ -8672,7 +8847,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>20:13:25</t>
+          <t>20:47:06</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -8686,7 +8861,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>79</v>
+        <v>45</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -8697,7 +8872,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>20:13:25</t>
+          <t>20:47:06</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -8711,7 +8886,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4114
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E253"/>
+  <dimension ref="A1:E260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:47:06</t>
+          <t>Última actualización: 21:36:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 248</t>
+          <t>Total filas: 255</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -833,7 +833,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>08:52:08</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:52:08</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>09:23:09</t>
+          <t>10:27:56</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>27</v>
+        <v>91</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>63</v>
+        <v>20</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>20</v>
+        <v>88</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -4073,7 +4073,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>14:51:15</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4083,11 +4083,11 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>72</v>
+        <v>15</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,7 +4098,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>14:51:15</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -4108,11 +4108,11 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>15</v>
+        <v>72</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>16:08:49</t>
+          <t>17:46:10</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5108,11 +5108,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>107</v>
+        <v>9</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>17:46:10</t>
+          <t>16:08:49</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>9</v>
+        <v>107</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>18:13:42</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>71</v>
+        <v>12</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>18:13:42</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>12</v>
+        <v>71</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -6473,7 +6473,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>20:47:06</t>
+          <t>21:36:27</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -6487,7 +6487,7 @@
         </is>
       </c>
       <c r="D246" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6498,12 +6498,12 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>20:13:25</t>
+          <t>21:36:27</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>21:42</t>
+          <t>21:40</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -6512,7 +6512,7 @@
         </is>
       </c>
       <c r="D247" t="n">
-        <v>89</v>
+        <v>4</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6523,12 +6523,12 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>20:47:06</t>
+          <t>20:13:25</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>21:50</t>
+          <t>21:42</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -6537,7 +6537,7 @@
         </is>
       </c>
       <c r="D248" t="n">
-        <v>63</v>
+        <v>89</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6553,16 +6553,16 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>21:59</t>
+          <t>21:50</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6573,21 +6573,21 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>20:47:06</t>
+          <t>21:36:27</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>22:07</t>
+          <t>21:59</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>80</v>
+        <v>23</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6598,21 +6598,21 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>20:47:06</t>
+          <t>21:36:27</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>22:26</t>
+          <t>21:59</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>99</v>
+        <v>23</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6628,16 +6628,16 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>22:37</t>
+          <t>22:07</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>110</v>
+        <v>80</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,23 +6648,198 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
+          <t>21:36:27</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>50</v>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>21:36:27</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>22:35</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D254" t="n">
+        <v>59</v>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>21:36:27</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D255" t="n">
+        <v>61</v>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>21:36:27</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>22:40</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D256" t="n">
+        <v>64</v>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
           <t>20:47:06</t>
         </is>
       </c>
-      <c r="B253" t="inlineStr">
+      <c r="B257" t="inlineStr">
         <is>
           <t>22:41</t>
         </is>
       </c>
-      <c r="C253" t="inlineStr">
+      <c r="C257" t="inlineStr">
         <is>
           <t>16_SANTA ANA</t>
         </is>
       </c>
-      <c r="D253" t="n">
+      <c r="D257" t="n">
         <v>114</v>
       </c>
-      <c r="E253" t="inlineStr">
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>21:36:27</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>22:55</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D258" t="n">
+        <v>79</v>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>21:36:27</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>23:07</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D259" t="n">
+        <v>91</v>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>21:36:27</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>23:29</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>113</v>
+      </c>
+      <c r="E260" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6681,7 +6856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6694,14 +6869,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:47:06</t>
+          <t>Última actualización: 21:36:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 45</t>
+          <t>Total filas: 46</t>
         </is>
       </c>
     </row>
@@ -7835,7 +8010,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>20:47:06</t>
+          <t>21:36:27</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -7849,9 +8024,34 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>110</v>
+        <v>61</v>
       </c>
       <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>21:36:27</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>23:29</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>113</v>
+      </c>
+      <c r="E51" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7881,7 +8081,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:47:06</t>
+          <t>Última actualización: 21:36:27</t>
         </is>
       </c>
     </row>
@@ -8872,7 +9072,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>20:47:06</t>
+          <t>21:36:27</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -8886,7 +9086,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>82</v>
+        <v>33</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4115
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-09.xlsx
+++ b/data/horarios-141-2026-08-09.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 21:36:27</t>
+          <t>Última actualización: 23:54:16</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -773,7 +773,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>07:20:43</t>
+          <t>06:07:50</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -783,11 +783,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>6</v>
+        <v>79</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>06:07:50</t>
+          <t>07:20:43</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>79</v>
+        <v>6</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>06:52:02</t>
+          <t>08:24:30</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>113</v>
+        <v>21</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>08:24:30</t>
+          <t>06:52:02</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>21</v>
+        <v>113</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>10:27:56</t>
+          <t>09:23:09</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>27</v>
+        <v>91</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>09:23:09</t>
+          <t>10:27:56</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>12:46:44</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>20</v>
+        <v>88</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>12:46:44</t>
+          <t>13:11:40</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>13:11:40</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>63</v>
+        <v>20</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -4073,7 +4073,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>14:51:15</t>
+          <t>13:54:42</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4083,11 +4083,11 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>15</v>
+        <v>72</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,7 +4098,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>13:54:42</t>
+          <t>14:51:15</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -4108,11 +4108,11 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>72</v>
+        <v>15</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4908,7 +4908,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -4933,7 +4933,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -5558,7 +5558,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D209" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5623,7 +5623,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>18:13:42</t>
+          <t>19:12:14</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -5633,11 +5633,11 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>63</v>
+        <v>4</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>19:12:14</t>
+          <t>18:13:42</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>4</v>
+        <v>63</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -6308,7 +6308,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D239" t="n">
@@ -6333,7 +6333,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D240" t="n">
@@ -6423,7 +6423,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>19:49:52</t>
+          <t>20:47:06</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -6433,11 +6433,11 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>107</v>
+        <v>49</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,7 +6448,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>20:47:06</t>
+          <t>19:49:52</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -6458,11 +6458,11 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>49</v>
+        <v>107</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6869,7 +6869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 21:36:27</t>
+          <t>Última actualización: 23:54:16</t>
         </is>
       </c>
     </row>
@@ -8081,7 +8081,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 21:36:27</t>
+          <t>Última actualización: 23:54:16</t>
         </is>
       </c>
     </row>

</xml_diff>